<commit_message>
Retrieved training dates and deployment timelines for 2025
</commit_message>
<xml_diff>
--- a/reference_files/2023_deployment_dates.xlsx
+++ b/reference_files/2023_deployment_dates.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Senior Year - College\Research\DataPullCode\PMDataCals\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Senior Year - College\Research\CalibrationCodes\Torrias2025Calibration\voz-data-analysis\reference_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{71222CEC-0430-445C-B80F-3FEB284B231D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA51D473-A6A2-48E9-B83A-1C85F128B009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DatesAvailable" sheetId="1" r:id="rId1"/>
-    <sheet name="2023_deployment_dates" sheetId="2" r:id="rId2"/>
+    <sheet name="Deployment Dates" sheetId="2" r:id="rId2"/>
     <sheet name="ExtendingCalibrationData" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -301,10 +301,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -6421,7 +6421,7 @@
         <v>36</v>
       </c>
       <c r="H3" s="6">
-        <f ca="1">OFFSET(DatesAvailable!B17,-'2023_deployment_dates'!F3*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!B17,-'Deployment Dates'!F3*0.2,0)</f>
         <v>45104</v>
       </c>
       <c r="I3" s="6">
@@ -6432,7 +6432,7 @@
         <v>45227</v>
       </c>
       <c r="K3" s="6">
-        <f ca="1">OFFSET(DatesAvailable!B122,'2023_deployment_dates'!G3*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!B122,'Deployment Dates'!G3*0.2,0)</f>
         <v>45239</v>
       </c>
       <c r="L3" t="s">
@@ -6532,7 +6532,7 @@
         <v>57</v>
       </c>
       <c r="H5" s="6">
-        <f ca="1">OFFSET(DatesAvailable!D31,-'2023_deployment_dates'!F5*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!D31,-'Deployment Dates'!F5*0.2,0)</f>
         <v>45107</v>
       </c>
       <c r="I5" s="6">
@@ -6542,7 +6542,7 @@
         <v>45233</v>
       </c>
       <c r="K5" s="6">
-        <f ca="1">OFFSET(DatesAvailable!D136,'2023_deployment_dates'!G5*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!D136,'Deployment Dates'!G5*0.2,0)</f>
         <v>45244</v>
       </c>
       <c r="L5" t="s">
@@ -6588,7 +6588,7 @@
         <v>26</v>
       </c>
       <c r="H6" s="6">
-        <f ca="1">OFFSET(DatesAvailable!E24,-'2023_deployment_dates'!F6*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!E24,-'Deployment Dates'!F6*0.2,0)</f>
         <v>45102</v>
       </c>
       <c r="I6" s="6">
@@ -6598,7 +6598,7 @@
         <v>45233</v>
       </c>
       <c r="K6" s="6">
-        <f ca="1">OFFSET(DatesAvailable!E127,'2023_deployment_dates'!G6*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!E127,'Deployment Dates'!G6*0.2,0)</f>
         <v>45247</v>
       </c>
       <c r="L6" t="s">
@@ -6646,7 +6646,7 @@
         <v>45227</v>
       </c>
       <c r="I7" s="6">
-        <f ca="1">OFFSET(DatesAvailable!F99,'2023_deployment_dates'!G7*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!F99,'Deployment Dates'!G7*0.2,0)</f>
         <v>45247</v>
       </c>
       <c r="J7" s="6">
@@ -6700,7 +6700,7 @@
         <v>31</v>
       </c>
       <c r="H8" s="6">
-        <f ca="1">OFFSET(DatesAvailable!G15,-'2023_deployment_dates'!F8*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!G15,-'Deployment Dates'!F8*0.2,0)</f>
         <v>45095</v>
       </c>
       <c r="I8" s="6">
@@ -6710,7 +6710,7 @@
         <v>45227</v>
       </c>
       <c r="K8" s="6">
-        <f ca="1">OFFSET(DatesAvailable!G132,'2023_deployment_dates'!G8*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!G132,'Deployment Dates'!G8*0.2,0)</f>
         <v>45238</v>
       </c>
       <c r="L8" t="s">
@@ -6756,7 +6756,7 @@
         <v>12</v>
       </c>
       <c r="H9" s="6">
-        <f ca="1">OFFSET(DatesAvailable!H16,-'2023_deployment_dates'!F9*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!H16,-'Deployment Dates'!F9*0.2,0)</f>
         <v>45095</v>
       </c>
       <c r="I9" s="6">
@@ -6766,7 +6766,7 @@
         <v>45233</v>
       </c>
       <c r="K9" s="6">
-        <f ca="1">OFFSET(DatesAvailable!H135,'2023_deployment_dates'!G9*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!H135,'Deployment Dates'!G9*0.2,0)</f>
         <v>45246</v>
       </c>
       <c r="L9" t="s">
@@ -6812,7 +6812,7 @@
         <v>30</v>
       </c>
       <c r="H10" s="6">
-        <f ca="1">OFFSET(DatesAvailable!I23,-'2023_deployment_dates'!F10*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!I23,-'Deployment Dates'!F10*0.2,0)</f>
         <v>45101</v>
       </c>
       <c r="I10" s="6">
@@ -6822,7 +6822,7 @@
         <v>45227</v>
       </c>
       <c r="K10" s="6">
-        <f ca="1">OFFSET(DatesAvailable!I112,'2023_deployment_dates'!G10*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!I112,'Deployment Dates'!G10*0.2,0)</f>
         <v>45238</v>
       </c>
       <c r="L10" t="s">
@@ -6868,7 +6868,7 @@
         <v>22</v>
       </c>
       <c r="H11" s="6">
-        <f ca="1">OFFSET(DatesAvailable!J24,-'2023_deployment_dates'!F11*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!J24,-'Deployment Dates'!F11*0.2,0)</f>
         <v>45115</v>
       </c>
       <c r="I11" s="6">
@@ -6878,7 +6878,7 @@
         <v>45244</v>
       </c>
       <c r="K11" s="6">
-        <f ca="1">OFFSET(DatesAvailable!J112,'2023_deployment_dates'!G11*0.2,0)</f>
+        <f ca="1">OFFSET(DatesAvailable!J112,'Deployment Dates'!G11*0.2,0)</f>
         <v>45248</v>
       </c>
       <c r="L11" t="s">

</xml_diff>

<commit_message>
Added demonstration folder for file input/output
</commit_message>
<xml_diff>
--- a/reference_files/2023_deployment_dates.xlsx
+++ b/reference_files/2023_deployment_dates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Senior Year - College\Research\CalibrationCodes\Torrias2025Calibration\voz-data-analysis\reference_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC977ED-A4C3-4A14-9625-ABD61D8BC5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D42F6E-1D14-4467-A41C-822DF09B4153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6397,8 +6397,8 @@
         <v>45231</v>
       </c>
       <c r="P2" s="6">
-        <f>E2</f>
-        <v>45291</v>
+        <f>E2+1</f>
+        <v>45292</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
@@ -6455,7 +6455,8 @@
         <v>45239</v>
       </c>
       <c r="P3" s="6">
-        <v>45249</v>
+        <f t="shared" ref="P3:P12" si="2">E3+1</f>
+        <v>45270</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
@@ -6513,8 +6514,8 @@
         <v>45238</v>
       </c>
       <c r="P4" s="6">
-        <f>DatesAvailable!C146</f>
-        <v>45269</v>
+        <f t="shared" si="2"/>
+        <v>45280</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
@@ -6570,6 +6571,7 @@
         <v>45244</v>
       </c>
       <c r="P5" s="6">
+        <f t="shared" si="2"/>
         <v>45292</v>
       </c>
     </row>
@@ -6626,6 +6628,7 @@
         <v>45247</v>
       </c>
       <c r="P6" s="6">
+        <f t="shared" si="2"/>
         <v>45292</v>
       </c>
     </row>
@@ -6682,6 +6685,7 @@
         <v>45247</v>
       </c>
       <c r="P7" s="6">
+        <f t="shared" si="2"/>
         <v>45281</v>
       </c>
     </row>
@@ -6738,6 +6742,7 @@
         <v>45238</v>
       </c>
       <c r="P8" s="6">
+        <f t="shared" si="2"/>
         <v>45280</v>
       </c>
     </row>
@@ -6794,6 +6799,7 @@
         <v>45246</v>
       </c>
       <c r="P9" s="6">
+        <f t="shared" si="2"/>
         <v>45270</v>
       </c>
     </row>
@@ -6850,6 +6856,7 @@
         <v>45238</v>
       </c>
       <c r="P10" s="6">
+        <f t="shared" si="2"/>
         <v>45292</v>
       </c>
     </row>
@@ -6906,6 +6913,7 @@
         <v>45248</v>
       </c>
       <c r="P11" s="6">
+        <f t="shared" si="2"/>
         <v>45280</v>
       </c>
     </row>
@@ -6960,8 +6968,8 @@
         <v>45231</v>
       </c>
       <c r="P12" s="6">
-        <f>E12</f>
-        <v>45291</v>
+        <f t="shared" si="2"/>
+        <v>45292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Can compare different kinds of calibrations for ozone now
</commit_message>
<xml_diff>
--- a/reference_files/2023_deployment_dates.xlsx
+++ b/reference_files/2023_deployment_dates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Senior Year - College\Research\CalibrationCodes\Torrias2025Calibration\voz-data-analysis\reference_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D42F6E-1D14-4467-A41C-822DF09B4153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217985C0-ADF9-4F86-A0DC-2A30F34332AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6447,7 +6447,7 @@
         <v>45092</v>
       </c>
       <c r="N3" s="6">
-        <f t="shared" ref="N3:N12" ca="1" si="0">H3</f>
+        <f t="shared" ref="N3:N11" ca="1" si="0">H3</f>
         <v>45104</v>
       </c>
       <c r="O3" s="6">
@@ -7148,7 +7148,7 @@
         <v>45092</v>
       </c>
       <c r="N3" s="6">
-        <f t="shared" ref="N3:N12" ca="1" si="0">H3</f>
+        <f t="shared" ref="N3:N11" ca="1" si="0">H3</f>
         <v>45104</v>
       </c>
       <c r="O3" s="6">
@@ -7850,7 +7850,7 @@
         <v>45104</v>
       </c>
       <c r="N3" s="6">
-        <f t="shared" ref="N3:N12" ca="1" si="1">H3</f>
+        <f t="shared" ref="N3:N11" ca="1" si="1">H3</f>
         <v>45104</v>
       </c>
       <c r="O3" s="6">

</xml_diff>